<commit_message>
ShiftMD Version 3.6 multilingual with additional shift type and ranked teams.
</commit_message>
<xml_diff>
--- a/demo-lekari.xlsx
+++ b/demo-lekari.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ShiftMD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{79795C07-F55B-42CB-A3E9-63656B5A2549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B5BDB822-0591-4B61-B949-B0F68033848F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="565" xr2:uid="{20F7004D-A330-4675-B7F7-3B4988869D2E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D3F95B20-AC2B-456A-8F7B-BCBAC4A8A1F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="52">
   <si>
     <t>Ime i prezime</t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t>Želi da dežura</t>
+  </si>
+  <si>
+    <t>Rang</t>
   </si>
   <si>
     <t>Dr Ana Antić</t>
@@ -198,16 +201,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -235,17 +230,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -586,393 +574,445 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39F53790-F83A-4524-954D-BF4153898131}">
-  <dimension ref="A1:G17"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B41EADF-4374-44D8-8880-BBCB260C0006}">
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.140625" customWidth="1"/>
-    <col min="2" max="2" width="18" style="3" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" customWidth="1"/>
-    <col min="6" max="6" width="23" style="5" customWidth="1"/>
-    <col min="7" max="7" width="24.85546875" style="5" customWidth="1"/>
+    <col min="1" max="1" width="20.42578125" customWidth="1"/>
+    <col min="2" max="2" width="16" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" customWidth="1"/>
+    <col min="6" max="6" width="24.85546875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="26" style="2" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="1">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="1">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="3">
+        <v>46301</v>
+      </c>
+      <c r="H3" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="3">
+        <v>46362</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="1">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="1">
         <v>7</v>
       </c>
-      <c r="B2" s="3">
-        <v>15</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C6" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+      <c r="D6" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="3">
+        <v>46240</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H6" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="1">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="1">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H8" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="1">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="3">
+        <v>46332</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="H9" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="1">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G10" s="3">
+        <v>46118</v>
+      </c>
+      <c r="H10" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="1">
+        <v>3</v>
+      </c>
+      <c r="C11" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="1">
+        <v>2</v>
+      </c>
+      <c r="C12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H12" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="1">
+        <v>2</v>
+      </c>
+      <c r="C13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" s="3">
+        <v>46271</v>
+      </c>
+      <c r="H13" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="1">
+        <v>1</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" t="s">
+        <v>33</v>
+      </c>
+      <c r="E14" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="3">
-        <v>12</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="6">
-        <v>46301</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="3">
-        <v>10</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="6">
-        <v>46362</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="3">
-        <v>8</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="3">
-        <v>7</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="6">
-        <v>46240</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="3">
-        <v>6</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" s="3">
+      <c r="G14" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H14" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="1">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G15" s="3">
+        <v>46332</v>
+      </c>
+      <c r="H15" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="1">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" t="s">
+        <v>33</v>
+      </c>
+      <c r="E16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H16" s="1">
         <v>5</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" t="s">
-        <v>26</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="3">
-        <v>4</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" t="s">
-        <v>26</v>
-      </c>
-      <c r="F9" s="6">
-        <v>46332</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="3">
-        <v>3</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" t="s">
-        <v>32</v>
-      </c>
-      <c r="E10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F10" s="5" t="s">
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" s="1">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" t="s">
         <v>33</v>
       </c>
-      <c r="G10" s="6">
-        <v>46118</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B11" s="3">
-        <v>3</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" t="s">
-        <v>15</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>36</v>
-      </c>
-      <c r="B12" s="3">
-        <v>2</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" t="s">
-        <v>32</v>
-      </c>
-      <c r="E12" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>39</v>
-      </c>
-      <c r="B13" s="3">
-        <v>2</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" t="s">
-        <v>21</v>
-      </c>
-      <c r="F13" s="6">
-        <v>46271</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>40</v>
-      </c>
-      <c r="B14" s="3">
+      <c r="E17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H17" s="1">
         <v>1</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" t="s">
-        <v>32</v>
-      </c>
-      <c r="E14" t="s">
-        <v>26</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15" s="3">
-        <v>1</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" t="s">
-        <v>32</v>
-      </c>
-      <c r="E15" t="s">
-        <v>26</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="G15" s="6">
-        <v>46332</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>44</v>
-      </c>
-      <c r="B16" s="3">
-        <v>1</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" t="s">
-        <v>32</v>
-      </c>
-      <c r="E16" t="s">
-        <v>45</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>48</v>
-      </c>
-      <c r="B17" s="3">
-        <v>1</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D17" t="s">
-        <v>32</v>
-      </c>
-      <c r="E17" t="s">
-        <v>45</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>